<commit_message>
Archive Project Spy and publish local training fixture
</commit_message>
<xml_diff>
--- a/docs/MAP.xlsx
+++ b/docs/MAP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Project-Spy\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCEEBE5F-0E30-424E-8870-D5EE8C5EC791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3010114B-F6B5-4F47-955B-C776C5518F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56FE8071-1488-4971-BCBC-5B907E79D7DF}"/>
   </bookViews>
@@ -81,10 +81,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>도로 (F)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>도로 (K)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -102,6 +98,10 @@
   </si>
   <si>
     <t>항구(충원)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">도로 </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -568,13 +568,13 @@
         <v>3</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.4">
@@ -582,7 +582,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>0</v>
@@ -624,7 +624,7 @@
         <v>5</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.4">
@@ -674,7 +674,7 @@
         <v>9</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.4">
@@ -1179,7 +1179,7 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>9</v>
@@ -1229,7 +1229,7 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>4</v>
@@ -1271,7 +1271,7 @@
         <v>1</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>3</v>
@@ -1279,13 +1279,13 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>3</v>

</xml_diff>